<commit_message>
Document the first live Jira+GitHub run in README and the delivery tracker
Records the B14 milestone: real sync/drift/brief run against a live team, the three
real bugs it surfaced and fixed (Jira /search/jql migration, Kanban board handling,
brief prompt placeholder leak), and that D1/D2 both verified firing on real data --
including organic activity from a second real team member. GO/NO-GO itself still
needs the lead's usefulness judgment, not something this tracker update can close.
</commit_message>
<xml_diff>
--- a/.claude/context/asof-delivery-tracker.xlsx
+++ b/.claude/context/asof-delivery-tracker.xlsx
@@ -2070,7 +2070,7 @@
       </c>
       <c r="F19" s="43" t="inlineStr">
         <is>
-          <t>CLI pipeline verified against fixtures; still needs real Jira/GitHub credentials + lead review to clear the GO/NO-GO gate</t>
+          <t>Real Jira Cloud site + real GitHub repo connected; sync/drift/brief run live end to end. D1 (KAN-16 Done w/ unmerged PR) and D2 (KAN-15/18/37 stale In Progress, 2 of them moved by a real second team member, Alex Cooper) both verified firing correctly. Still needs: your own usefulness judgment on the findings to actually clear the GO/NO-GO gate.</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="I18" s="43" t="inlineStr">
         <is>
-          <t>src/cli/{sync,drift,brief}.ts built and verified end-to-end against real local Postgres, incl. auto-resolve (test/fixtures/demoTeam.ts, ASOF_DEMO_PHASE=1/2). NOT done: the actual GO/NO-GO gate needs a real team's Jira+GitHub data and a lead's usefulness judgment -- neither is something this session can perform. Next: point .env at a real Jira project + GitHub repo and run the 3 commands for real.</t>
+          <t>First real sync+drift+brief run completed against a real Jira Cloud site (KAN project) + real GitHub repo (vinaycookscode/AsOf), with a second real team member (Alex Cooper) independently active on the board. Fixed 3 real bugs the live run surfaced: Jira's /rest/api/3/search was removed (migrated to /rest/api/3/search/jql, cursor pagination); fetchActiveSprint crashed on Kanban boards (400 'board does not support sprints') instead of treating it as sprint=null; brief prompt leaked a literal 'Sprint day X of Y' placeholder when sprint was null. D1 and D2 both verified firing correctly on real data (issues transitioned via the Jira API directly, since CSV-imported issues have no changelog history for their seeded status). STILL NOT DONE: the actual GO/NO-GO judgment call -- are these findings useful -- is the user's to make, not something this session can perform.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B19: Fuzzy PR<->ticket matching via Haiku
Last-resort linking pass for PRs no rule-based source matched. Opt-in (only runs
when ANTHROPIC_API_KEY is set, only on PRs nothing else already linked), always
linkSource "fuzzy" so it can never drive a High-severity finding per the existing
D1/D2/D6 linking gate. 9 fixture tests against a mocked linker client.
</commit_message>
<xml_diff>
--- a/.claude/context/asof-delivery-tracker.xlsx
+++ b/.claude/context/asof-delivery-tracker.xlsx
@@ -2148,7 +2148,7 @@
       </c>
       <c r="D22" s="43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E22" s="43" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="F22" s="43" t="inlineStr">
         <is>
-          <t>Highest technical risk - do early</t>
+          <t>Explicit (B7) + branch/commit-ref (B8) + fuzzy via Haiku (B19), all fixture-tested.</t>
         </is>
       </c>
     </row>
@@ -3706,10 +3706,14 @@
       </c>
       <c r="H23" s="43" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I23" s="43" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I23" s="43" t="inlineStr">
+        <is>
+          <t>src/linking/fuzzy.ts -- extractFuzzyLinks() only calls Haiku for PRs no rule-based source matched, offers the connected project's issue titles as candidates, discards &lt;0.5 confidence and any hallucinated key not in the offered list. linkSource always 'fuzzy' -- D1/D2/D6 already exclude fuzzy from their linking gate (drift-rules-spec.md), so this can only ever support Medium/Low findings, never drive a High one. Wired into resolveLinksWithFuzzy()/cli/sync.ts as opt-in: only runs when ANTHROPIC_API_KEY is set, otherwise npm run sync stays on the existing synchronous rule-based-only path. 9 fixture tests (TP/boundary/FP-trap/resolution + prompt-parsing edge cases) against a mocked FuzzyLinkerClient, no live API calls in CI.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="24">
       <c r="A24" s="41" t="inlineStr">

</xml_diff>

<commit_message>
B26: Per-team rule config API + workflow status mapping
Wires up the existing (previously unused) rule_config table via GET/PUT
/api/settings/rules/:ruleId -- per-team enabled/params/slackDelivery, merged onto
the drift-rules-spec.md defaults. drift.ts now loads this instead of the hardcoded
DEFAULT_RULE_CONFIG, filtering disabled rules' findings before persisting (which
auto-resolves their previously-open findings via B25's lifecycle, free).

Also adds team.status_category_map + GET/PUT /api/settings/status-map for the
onboarding workflow-mapping step, closing the loop on a JiraClient constructor
param that existed since B3 but nothing ever persisted or fed.

Verified live against the real KAN team: disabled D2, findings auto-resolved;
raised its threshold, confirmed suppression; reset to defaults, findings reopened
in place without duplicating.
</commit_message>
<xml_diff>
--- a/.claude/context/asof-delivery-tracker.xlsx
+++ b/.claude/context/asof-delivery-tracker.xlsx
@@ -2180,7 +2180,7 @@
       </c>
       <c r="D23" s="43" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E23" s="43" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="F23" s="43" t="inlineStr">
         <is>
-          <t>All 8 rules (D1-D8) implemented and fixture-tested (B10-B12, B20-B24). Per-team rule config API (B26) not started.</t>
+          <t>All 8 rules (B10-B12, B20-B24) + per-team rule config API (B26), all verified live against real Jira data.</t>
         </is>
       </c>
     </row>
@@ -4035,10 +4035,14 @@
       </c>
       <c r="H30" s="43" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I30" s="43" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I30" s="43" t="inlineStr">
+        <is>
+          <t>src/db/ruleConfig.ts + src/api/routes/settings.ts. GET/PUT /api/settings/rules/:ruleId reads/writes the existing (previously unused) rule_config table -- enabled/params/slackDelivery merged onto drift-rules-spec.md defaults. cli/drift.ts now loads per-team config instead of hardcoded DEFAULT_RULE_CONFIG and filters disabled rules' findings before persisting (which auto-resolves their previously-open findings for free via B25's lifecycle). Also added team.status_category_map (migration 003) + GET/PUT /api/settings/status-map for the onboarding workflow-mapping step (design-spec.md 2.1); cli/sync.ts loads it before constructing JiraClient. No onboarding UI writes to it yet (B15/B34). Verified live against the real KAN team: disabled D2 via the API, findings correctly auto-resolved (not deleted); raised d2.days to 10, confirmed suppression; reset to defaults, findings reopened in place without duplicating.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="23.25" customHeight="1" s="24">
       <c r="A31" s="41" t="inlineStr">

</xml_diff>